<commit_message>
Live Supabase Results added & Synched
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/JSS3/Mathematics/results.xlsx
+++ b/RESULTS/2017/CLASS/JSS3/Mathematics/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,6 +465,52 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>Submitted At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Adetoye Haneefah Aderinsola</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>std98</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JSS3</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:06:13.831Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ca test, Atendance & Exam Page Re-designed
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/JSS3/Mathematics/results.xlsx
+++ b/RESULTS/2017/CLASS/JSS3/Mathematics/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,11 +491,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>50</v>
@@ -506,11 +506,149 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-22T13:06:13.831Z</t>
+          <t>2026-06-04T07:59:04.188Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Abdulrasheed Yusrah</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>std89</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>JSS3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>64</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-06-05T09:38:35.501Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jibril Fatima Zara</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>std93</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>JSS3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>38</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-06-05T09:40:13.285Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aliyu Zainab Musa</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>std85</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>JSS3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>14</v>
+      </c>
+      <c r="G5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>51</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-06-05T09:41:50.020Z</t>
         </is>
       </c>
     </row>

</xml_diff>